<commit_message>
verification updatre issue fixed
</commit_message>
<xml_diff>
--- a/AdvanceCRM/AdvanceCRM.Web/Templates/DemandaySpecs_Template.xlsx
+++ b/AdvanceCRM/AdvanceCRM.Web/Templates/DemandaySpecs_Template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Sr No</t>
   </si>
@@ -36,6 +36,9 @@
   </si>
   <si>
     <t>Annual Revenue</t>
+  </si>
+  <si>
+    <t>Exclude Company</t>
   </si>
   <si>
     <t>Address</t>
@@ -108,7 +111,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -119,13 +122,14 @@
     <col min="6" max="6" width="22" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
     <col min="8" max="8" width="20" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
     <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="10" customWidth="1"/>
-    <col min="12" max="12" width="12" customWidth="1"/>
-    <col min="13" max="13" width="20" customWidth="1"/>
+    <col min="11" max="11" width="12" customWidth="1"/>
+    <col min="12" max="12" width="10" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="20" customWidth="1"/>
     <col min="15" max="15" width="20" customWidth="1"/>
+    <col min="16" max="16" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -174,6 +178,9 @@
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <headerFooter/>

</xml_diff>